<commit_message>
KIBONBE-229: Rename variable Refactor sum calculation excel
</commit_message>
<xml_diff>
--- a/ebegu-server/src/main/resources/reporting/Gemeinden.xlsx
+++ b/ebegu-server/src/main/resources/reporting/Gemeinden.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\new\ebegu\ebegu-server\src\main\resources\reporting\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soja\Documents\projects\kibon-app\ebegu-server\src\main\resources\reporting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37766289-53A3-48D7-9D26-60DDB7E5847A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1A404F-364C-43CC-9210-9596C71C4F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Angaben pro Gemeinde" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>{gemeindenTitle}</t>
   </si>
@@ -137,6 +137,48 @@
   </si>
   <si>
     <t>{gemeindeKennzahlenStatus}</t>
+  </si>
+  <si>
+    <t>{gemeindeGueltigBis}</t>
+  </si>
+  <si>
+    <t>{gemeindeGueltigBisTitle}</t>
+  </si>
+  <si>
+    <t>{eMailStammdatenTitle}</t>
+  </si>
+  <si>
+    <t>{eMailStammdaten}</t>
+  </si>
+  <si>
+    <t>{phoneStammdatenTitle}</t>
+  </si>
+  <si>
+    <t>{phoneStammdaten}</t>
+  </si>
+  <si>
+    <t>{eMailBGTitle}</t>
+  </si>
+  <si>
+    <t>{eMailBG}</t>
+  </si>
+  <si>
+    <t>{phoneBGTitle}</t>
+  </si>
+  <si>
+    <t>{phoneBG}</t>
+  </si>
+  <si>
+    <t>{eMailTSATitle}</t>
+  </si>
+  <si>
+    <t>{eMailTSA}</t>
+  </si>
+  <si>
+    <t>{phoneTSATitle}</t>
+  </si>
+  <si>
+    <t>{phoneTSA}</t>
   </si>
 </sst>
 </file>
@@ -522,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F97ADB9F-B7F2-409A-AE88-F2E4D15479F3}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -531,23 +573,30 @@
     <col min="4" max="4" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.42578125" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="49.42578125" customWidth="1"/>
+    <col min="10" max="10" width="24.7109375" customWidth="1"/>
+    <col min="11" max="11" width="49.42578125" customWidth="1"/>
+    <col min="12" max="12" width="29.28515625" customWidth="1"/>
+    <col min="13" max="13" width="49.42578125" customWidth="1"/>
+    <col min="14" max="14" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>2</v>
       </c>
@@ -569,8 +618,29 @@
       <c r="G5" s="9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -578,8 +648,15 @@
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -587,8 +664,15 @@
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -610,12 +694,40 @@
       <c r="G8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="O8" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="14">
+    <mergeCell ref="N5:N7"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="L5:L7"/>
+    <mergeCell ref="M5:M7"/>
+    <mergeCell ref="H5:H7"/>
     <mergeCell ref="G5:G7"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
@@ -625,6 +737,7 @@
     <mergeCell ref="F5:F7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -637,13 +750,14 @@
     <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" customWidth="1"/>
+    <col min="5" max="5" width="39.42578125" customWidth="1"/>
     <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.42578125" customWidth="1"/>
+    <col min="12" max="12" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
@@ -673,7 +787,7 @@
         <v>19</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>21</v>
@@ -688,10 +802,10 @@
         <v>27</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -707,8 +821,8 @@
       <c r="D6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>36</v>
+      <c r="E6" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>22</v>
@@ -722,11 +836,11 @@
       <c r="I6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>30</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="L6" t="s">
         <v>31</v>

</xml_diff>